<commit_message>
Fix unalligned answers precise_ta, need to add translations to 2 missing ans in hi/ta, also update a golden answer to include tanglish
</commit_message>
<xml_diff>
--- a/datasets/IndicWikiQA-Tam_EN.xlsx
+++ b/datasets/IndicWikiQA-Tam_EN.xlsx
@@ -268,7 +268,7 @@
     <t>What is the simple, thick boiled lentil preparation often mixed with rice and ghee at the beginning of a traditional Tamil meal?</t>
   </si>
   <si>
-    <t>Dal</t>
+    <t>Dal (Paruppu)</t>
   </si>
   <si>
     <t>https://en.wikipedia.org/wiki/Dal</t>
@@ -4873,7 +4873,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75">
       <c r="A184" s="2" t="s">
         <v>519</v>
       </c>
@@ -4887,7 +4887,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75">
       <c r="A185" s="2" t="s">
         <v>521</v>
       </c>
@@ -4901,7 +4901,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75">
       <c r="A186" s="2" t="s">
         <v>524</v>
       </c>
@@ -4915,7 +4915,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75">
       <c r="A187" s="2" t="s">
         <v>527</v>
       </c>
@@ -4929,7 +4929,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75">
       <c r="A188" s="2" t="s">
         <v>530</v>
       </c>
@@ -4943,7 +4943,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75">
       <c r="A189" s="2" t="s">
         <v>533</v>
       </c>
@@ -4957,7 +4957,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75">
       <c r="A190" s="2" t="s">
         <v>536</v>
       </c>
@@ -4971,7 +4971,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75">
       <c r="A191" s="2" t="s">
         <v>539</v>
       </c>
@@ -4985,7 +4985,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75">
       <c r="A192" s="2" t="s">
         <v>542</v>
       </c>
@@ -4999,7 +4999,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75">
       <c r="A193" s="2" t="s">
         <v>545</v>
       </c>
@@ -5013,7 +5013,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75">
       <c r="A194" s="2" t="s">
         <v>548</v>
       </c>
@@ -5027,7 +5027,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75">
       <c r="A195" s="2" t="s">
         <v>551</v>
       </c>
@@ -5041,7 +5041,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75">
       <c r="A196" s="2" t="s">
         <v>554</v>
       </c>
@@ -5055,7 +5055,7 @@
         <v>287</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75">
       <c r="A197" s="2" t="s">
         <v>557</v>
       </c>

</xml_diff>